<commit_message>
Word a Excel: doplněno 1. trojročí, výstupy přegenerovány
Kontrola odhalila dvě věci:

1) Word vypisoval v Diferenciaci jen 2. a 3. trojročí — dif1 se do
   build_docx.js nikdy nedoplnil, přidalo se jen do webu. Opraveno;
   téma 40 správně vypíše 1. a 3. (dif2 má prázdné).

2) Soubory ve vystupy/ byly zastaralé — obsahovaly 48x '2 i 3' a 2x
   'jen 3.', tedy stav PŘED otevřením tématu 26 druhému trojročí i před
   změnou modelu urovne. Nebyly přegenerované od začátku srpna.

Po přegenerování: Excel 49x '1.–3.' + 1x 'jen 3.', Word 49x
'1.–3. trojročí' + 1x 'jen 3. trojročí', diferenciace 1./2./3. u 50/49/50
témat (2. chybí jen u tématu 40, kde je prázdná záměrně).

Excel diferenciace neobsahuje vůbec — je to přehledová tabulka pro výběr
témat (sloupec 'Kdo si téma bere'), ne metodika; doplňuje se jen sloupec
Trojročí.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/vystupy/Projektova_temata.xlsx
+++ b/vystupy/Projektova_temata.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Témata" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pokrytí kamenů" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Jak s tabulkou pracovat" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Témata" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Pokrytí kamenů" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Jak s tabulkou pracovat" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Témata'!$A$1:$K$51</definedName>
@@ -608,7 +608,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>2 i 3</t>
+          <t>1.–3.</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
@@ -669,7 +669,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>2 i 3</t>
+          <t>1.–3.</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
@@ -731,7 +731,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>2 i 3</t>
+          <t>1.–3.</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
@@ -792,7 +792,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>2 i 3</t>
+          <t>1.–3.</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -854,7 +854,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>2 i 3</t>
+          <t>1.–3.</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
@@ -915,7 +915,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>2 i 3</t>
+          <t>1.–3.</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
@@ -977,7 +977,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>2 i 3</t>
+          <t>1.–3.</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
@@ -1039,7 +1039,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>2 i 3</t>
+          <t>1.–3.</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -1099,7 +1099,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>2 i 3</t>
+          <t>1.–3.</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
@@ -1166,7 +1166,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>2 i 3</t>
+          <t>1.–3.</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
@@ -1230,7 +1230,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>2 i 3</t>
+          <t>1.–3.</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr">
@@ -1291,7 +1291,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>2 i 3</t>
+          <t>1.–3.</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
@@ -1352,7 +1352,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>2 i 3</t>
+          <t>1.–3.</t>
         </is>
       </c>
       <c r="G14" s="3" t="inlineStr">
@@ -1413,7 +1413,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>2 i 3</t>
+          <t>1.–3.</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
@@ -1474,7 +1474,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>2 i 3</t>
+          <t>1.–3.</t>
         </is>
       </c>
       <c r="G16" s="3" t="inlineStr">
@@ -1535,7 +1535,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>2 i 3</t>
+          <t>1.–3.</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
@@ -1597,7 +1597,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>2 i 3</t>
+          <t>1.–3.</t>
         </is>
       </c>
       <c r="G18" s="3" t="inlineStr">
@@ -1660,7 +1660,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>2 i 3</t>
+          <t>1.–3.</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -1721,7 +1721,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>2 i 3</t>
+          <t>1.–3.</t>
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr">
@@ -1782,7 +1782,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>2 i 3</t>
+          <t>1.–3.</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
@@ -1844,7 +1844,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>2 i 3</t>
+          <t>1.–3.</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr">
@@ -1905,7 +1905,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>2 i 3</t>
+          <t>1.–3.</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
@@ -1967,7 +1967,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>2 i 3</t>
+          <t>1.–3.</t>
         </is>
       </c>
       <c r="G24" s="3" t="inlineStr">
@@ -2029,7 +2029,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>2 i 3</t>
+          <t>1.–3.</t>
         </is>
       </c>
       <c r="G25" s="3" t="inlineStr">
@@ -2091,7 +2091,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>2 i 3</t>
+          <t>1.–3.</t>
         </is>
       </c>
       <c r="G26" s="3" t="inlineStr">
@@ -2154,7 +2154,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>jen 3.</t>
+          <t>1.–3.</t>
         </is>
       </c>
       <c r="G27" s="3" t="inlineStr">
@@ -2215,7 +2215,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>2 i 3</t>
+          <t>1.–3.</t>
         </is>
       </c>
       <c r="G28" s="3" t="inlineStr">
@@ -2278,7 +2278,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>2 i 3</t>
+          <t>1.–3.</t>
         </is>
       </c>
       <c r="G29" s="3" t="inlineStr">
@@ -2340,7 +2340,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>2 i 3</t>
+          <t>1.–3.</t>
         </is>
       </c>
       <c r="G30" s="3" t="inlineStr">
@@ -2400,7 +2400,7 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>2 i 3</t>
+          <t>1.–3.</t>
         </is>
       </c>
       <c r="G31" s="3" t="inlineStr">
@@ -2462,7 +2462,7 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>2 i 3</t>
+          <t>1.–3.</t>
         </is>
       </c>
       <c r="G32" s="3" t="inlineStr">
@@ -2524,7 +2524,7 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>2 i 3</t>
+          <t>1.–3.</t>
         </is>
       </c>
       <c r="G33" s="3" t="inlineStr">
@@ -2586,7 +2586,7 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>2 i 3</t>
+          <t>1.–3.</t>
         </is>
       </c>
       <c r="G34" s="3" t="inlineStr">
@@ -2648,7 +2648,7 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>2 i 3</t>
+          <t>1.–3.</t>
         </is>
       </c>
       <c r="G35" s="3" t="inlineStr">
@@ -2711,7 +2711,7 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>2 i 3</t>
+          <t>1.–3.</t>
         </is>
       </c>
       <c r="G36" s="3" t="inlineStr">
@@ -2775,7 +2775,7 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>2 i 3</t>
+          <t>1.–3.</t>
         </is>
       </c>
       <c r="G37" s="3" t="inlineStr">
@@ -2836,7 +2836,7 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>2 i 3</t>
+          <t>1.–3.</t>
         </is>
       </c>
       <c r="G38" s="3" t="inlineStr">
@@ -2898,7 +2898,7 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>2 i 3</t>
+          <t>1.–3.</t>
         </is>
       </c>
       <c r="G39" s="3" t="inlineStr">
@@ -2959,7 +2959,7 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>2 i 3</t>
+          <t>1.–3.</t>
         </is>
       </c>
       <c r="G40" s="3" t="inlineStr">
@@ -3084,7 +3084,7 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>2 i 3</t>
+          <t>1.–3.</t>
         </is>
       </c>
       <c r="G42" s="3" t="inlineStr">
@@ -3146,7 +3146,7 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>2 i 3</t>
+          <t>1.–3.</t>
         </is>
       </c>
       <c r="G43" s="3" t="inlineStr">
@@ -3208,7 +3208,7 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>2 i 3</t>
+          <t>1.–3.</t>
         </is>
       </c>
       <c r="G44" s="3" t="inlineStr">
@@ -3270,7 +3270,7 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>2 i 3</t>
+          <t>1.–3.</t>
         </is>
       </c>
       <c r="G45" s="3" t="inlineStr">
@@ -3333,7 +3333,7 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>2 i 3</t>
+          <t>1.–3.</t>
         </is>
       </c>
       <c r="G46" s="3" t="inlineStr">
@@ -3395,7 +3395,7 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>2 i 3</t>
+          <t>1.–3.</t>
         </is>
       </c>
       <c r="G47" s="3" t="inlineStr">
@@ -3457,7 +3457,7 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>2 i 3</t>
+          <t>1.–3.</t>
         </is>
       </c>
       <c r="G48" s="3" t="inlineStr">
@@ -3519,7 +3519,7 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>2 i 3</t>
+          <t>1.–3.</t>
         </is>
       </c>
       <c r="G49" s="3" t="inlineStr">
@@ -3581,7 +3581,7 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>2 i 3</t>
+          <t>1.–3.</t>
         </is>
       </c>
       <c r="G50" s="3" t="inlineStr">
@@ -3644,7 +3644,7 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>2 i 3</t>
+          <t>1.–3.</t>
         </is>
       </c>
       <c r="G51" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Doplnit dif1/aktivity/znalosti u témat 17, 19, 41, 43 podle návrhu kolegyně
Reakce na návrhy témat pro 1. trojročí (Místo, kde žijeme; Lidé a čas I;
Rozmanitost přírody I): státní symboly a vlast u tématu 43, orientace na
mapě ČR u tématu 19, regionální pověsti u tématu 17, půda a koloběh vody
u tématu 41. Přegenerováno index.html, Word i Excel.
</commit_message>
<xml_diff>
--- a/vystupy/Projektova_temata.xlsx
+++ b/vystupy/Projektova_temata.xlsx
@@ -1609,7 +1609,7 @@
         <is>
           <t>• Detektivka nad pramenem: co prozradí stará fotografie, mince, kronika či dopis z fronty — čtení a interpretace pramenů
 • Návštěva archivu, muzea či knihovny se zadáním: najít odpověď na vlastní historickou otázku
-• Historie místa: pátrání po minulosti školy, ulice či obce (staré mapy, pamětní desky, katastr, kroniky)
+• Historie místa: pátrání po minulosti školy, ulice či obce (staré mapy, pamětní desky, katastr, kroniky, místní pověsti a legendy)
 • Rozhovor s pamětníkem (metoda orální historie) a jeho porovnání s písemnými zdroji — kde se liší a proč
 • Výstava či podcast „Stopy minulosti“: děti prezentují svá zjištění s uvedením pramenů</t>
         </is>
@@ -1620,7 +1620,8 @@
 • Dějepis: posoudí informační hodnotu a důvěryhodnost zdrojů z různých dějinných epoch (přímý OVU revize!); rozdíl mezi dějepisectvím a zobrazením v médiích
 • Český jazyk a literatura: čtení s porozuměním, práce s věcným i uměleckým textem
 • Geografie: staré mapy a proměny krajiny
-• Informatika: digitální archivy, vyhledávání a hodnocení informací</t>
+• Informatika: digitální archivy, vyhledávání a hodnocení informací
+• Český jazyk a literatura: pověsti a legendy jako lidový pramen paměti místa</t>
         </is>
       </c>
       <c r="J18" s="3" t="inlineStr">
@@ -1735,7 +1736,8 @@
 • Mapová dílna: čtení map, práce s měřítkem, plánování trasy, tvorba mapy okolí školy či vlastního „mentálního území“
 • Grafová dílna: stejná data, různé grafy — kdy který použít a jak grafy klamou
 • Orientační výprava městem jen podle plánů, řádů a schémat MHD
-• Tvorba infografiky na zvolené téma pro školní chodbu</t>
+• Tvorba infografiky na zvolené téma pro školní chodbu
+• Mapa ČR poprvé: kde jsme, jaké kraje má naše země a kdo jsou naši sousedé</t>
         </is>
       </c>
       <c r="I20" s="3" t="inlineStr">
@@ -1743,7 +1745,8 @@
           <t>• grafy a proměnné, mapy a mapové symboly, kódování (piktogramy, symboly), obrazové modely (myšlenkové mapy, schémata, tabulky); (Ú3) grafy s více proměnnými, bit a bajt, jednoduché šifry, vývojové diagramy
 • Geografie: kriticky využívá mapy a zdroje geografických dat; geoinformační technologie
 • Matematika: diagramy, grafy, tabulky; měřítko a poměr
-• Informatika: kódování dat, odvození informací z modelu</t>
+• Informatika: kódování dat, odvození informací z modelu
+• Člověk a jeho svět: orientace na mapě ČR a Evropy, sousední státy</t>
         </is>
       </c>
       <c r="J20" s="3" t="inlineStr">
@@ -3098,7 +3101,8 @@
 • Experiment „les vs. obrazovka“: měření nálady a soustředění po hodině venku a po hodině u obrazovky
 • Tiché techniky venku: sedové místo (sit spot), smyslové vnímání, deník pozorování přírody
 • Adopce kousku přírody: dlouhodobá péče o strom, tůňku či záhon v okolí školy, úklidová akce
-• Beseda s ekologem či ochranářem, exkurze do CHKO nebo záchranné stanice</t>
+• Beseda s ekologem či ochranářem, exkurze do CHKO nebo záchranné stanice
+• Cesta kapky vody: pozorování a pokusy s koloběhem vody a půdou v okolí školy (louže, pára, sníh, propustnost půdy)</t>
         </is>
       </c>
       <c r="I42" s="3" t="inlineStr">
@@ -3107,7 +3111,8 @@
 • Geografie: krajina a její typy, chráněná území, udržitelnost
 • Výchova ke zdraví a bezpečí: duševní hygiena, rovnováha zátěže a odpočinku
 • Osobnostní a sociální výchova: všímá si svého prožívání, postupy předcházení stresu
-• relaxační techniky; formy odpočinku, které mi fungují</t>
+• relaxační techniky; formy odpočinku, které mi fungují
+• Přírodopis: půda a její vlastnosti, koloběh vody v přírodě</t>
         </is>
       </c>
       <c r="J42" s="3" t="inlineStr">
@@ -3222,7 +3227,8 @@
 • Tři moci v akci: hra na zákonodárce, vládu a soud — proč se moc dělí a co se stane, když ne
 • Návštěva jednání obecního zastupitelstva, radnice či Poslanecké sněmovny; rozhovor se zastupitelem
 • Mapa institucí: kdo mi vydá občanku, kdo opravuje silnici, kdo mě soudí, co dělá EU/NATO/OSN — a kam se obrátit se skutečným podnětem
-• Občanský projekt naostro: podnět či petice k reálnému problému v okolí školy (přechod, hřiště, koš)</t>
+• Občanský projekt naostro: podnět či petice k reálnému problému v okolí školy (přechod, hřiště, koš)
+• Vlajka, znak a hymna: co znamenají státní symboly a proč je máme; procházka obcí za pamětihodnostmi jako symboly domova</t>
         </is>
       </c>
       <c r="I44" s="3" t="inlineStr">
@@ -3231,7 +3237,8 @@
 • Dějepis: vznik moderních států a demokracie
 • Geografie: státy a jejich integrace, konfliktní ohniska světa
 • Český jazyk a literatura: úřední komunikace — podnět, petice, žádost
-• Matematika: volební aritmetika — poměrné rozdělení mandátů, procenta</t>
+• Matematika: volební aritmetika — poměrné rozdělení mandátů, procenta
+• Člověk a jeho svět: domov, škola a okolí, obec a vlast, základní státní symboly (vlajka, znak, hymna)</t>
         </is>
       </c>
       <c r="J44" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Rozšířit témata 42 a 43 podle druhé dávky nápadů kolegů
Téma 42 (Století extrémů) doplněno o prožitkovou aktivitu s dobovými
praktickými dovednostmi (praní, zašívání, ladění rádia) podle návrhu
„Krvavé století: jak žily naše prababičky". Téma 43 (Stát a my) doplněno
o aktivitu umožňující mimořádné zařazení projektu v čase skutečných voleb.
Přegenerováno index.html, Word i Excel.
</commit_message>
<xml_diff>
--- a/vystupy/Projektova_temata.xlsx
+++ b/vystupy/Projektova_temata.xlsx
@@ -3165,7 +3165,8 @@
 • Práce s pamětnickými nahrávkami (Paměť národa) a pozvání pamětníka do školy
 • Rozbor propagandy: dobové plakáty, týdeníky a noviny — jak se vyrábí nepřítel; paralely s dnešní manipulací
 • Příběhy odvahy a selhání: Wintonovy děti, bratři Mašínové, Charta 77 — diskuse o hranicích odvahy a přizpůsobení
-• Exkurze: Terezín, Vojna u Příbrami, Muzeum paměti XX. století či místní místa paměti</t>
+• Exkurze: Terezín, Vojna u Příbrami, Muzeum paměti XX. století či místní místa paměti
+• Den jako prababička: praktické dovednosti všedního dne (praní v kolíbce, zašívání, ladění rádia, vaření z tehdejších surovin) jako zážitková sonda do doby</t>
         </is>
       </c>
       <c r="I43" s="3" t="inlineStr">
@@ -3174,7 +3175,8 @@
 • Výchova k občanství: demokratická vs. autokratická vláda a jejich dopady na život občanů; lidská práva
 • Český jazyk a literatura: rozpoznává manipulaci, kriticky posuzuje mediální sdělení
 • Geografie: proměny hranic a migrace ve 20. století
-• manipulativní chování a techniky, jak mu čelit; dezinformační kampaně</t>
+• manipulativní chování a techniky, jak mu čelit; dezinformační kampaně
+• Polytechnická výchova a praktické činnosti: běžné domácí práce dřívějška (praní, šití, drobné opravy) jako zážitková sonda do každodennosti minulosti</t>
         </is>
       </c>
       <c r="J43" s="3" t="inlineStr">
@@ -3228,7 +3230,8 @@
 • Návštěva jednání obecního zastupitelstva, radnice či Poslanecké sněmovny; rozhovor se zastupitelem
 • Mapa institucí: kdo mi vydá občanku, kdo opravuje silnici, kdo mě soudí, co dělá EU/NATO/OSN — a kam se obrátit se skutečným podnětem
 • Občanský projekt naostro: podnět či petice k reálnému problému v okolí školy (přechod, hřiště, koš)
-• Vlajka, znak a hymna: co znamenají státní symboly a proč je máme; procházka obcí za pamětihodnostmi jako symboly domova</t>
+• Vlajka, znak a hymna: co znamenají státní symboly a proč je máme; procházka obcí za pamětihodnostmi jako symboly domova
+• Mimořádné zařazení podle kalendáře: konají-li se skutečné volby (prezidentské, parlamentní, komunální), lze projekt zařadit i mimo plánovaný blok, aby ho děti zažily v reálném čase</t>
         </is>
       </c>
       <c r="I44" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Nové téma 51 Čtení tě mění (SC1, jen 3. trojročí)
Podle návrhu kolegyně na čtenářské strategie a výběr knih. Omezeno na
3. trojročí — 1. a 2. trojročí už čtenářské strategie řeší v pravidelné
čtenářské dílně, takže samostatný projekt nepotřebují (stejný vzorec jako
u tématu 40 Právo pro život). Katalog má nyní 51 témat, README aktualizováno,
přegenerováno index.html, Word i Excel.
</commit_message>
<xml_diff>
--- a/vystupy/Projektova_temata.xlsx
+++ b/vystupy/Projektova_temata.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Jak s tabulkou pracovat" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Témata'!$A$1:$K$51</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Témata'!$A$1:$K$52</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Pokrytí kamenů'!$A$1:$H$121</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -507,7 +507,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K51"/>
+  <dimension ref="A1:K52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3688,8 +3688,68 @@
       </c>
       <c r="K51" s="3" t="inlineStr"/>
     </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>Čtení tě mění</t>
+        </is>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>SC1 Umím se učit</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>1.1.2.1 Čtu a naslouchám</t>
+        </is>
+      </c>
+      <c r="E52" s="3" t="inlineStr">
+        <is>
+          <t>1.1.1.2 Vyhledám relevantní zdroj učení
+1.2.4.4 Přetavuji prožitky ve zkušenosti
+1.1.2.9 Učím se skrze umění
+5.3.1.3 Vyjadřuji se písemně</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>jen 3.</t>
+        </is>
+      </c>
+      <c r="G52" s="3" t="inlineStr">
+        <is>
+          <t>Kniha, která k tobě promluví, dokáže změnit, jak myslíš a jak žiješ. Projekt je čtenářskou dílnou: děti se učí vybírat si knihy podle sebe, zkoušejí různé čtenářské strategie (předvídání, vizualizace, spojování s vlastním životem) a hledají v příbězích postavy a situace, které jim pomáhají porozumět vlastnímu životu. Čtení tu není povinnost, ale nástroj poznání sebe i světa.</t>
+        </is>
+      </c>
+      <c r="H52" s="3" t="inlineStr">
+        <is>
+          <t>• Čtenářský profil: jaký jsem typ čtenáře — žánry, tempo, kde a kdy se mi čte nejlépe; sestavení osobního čtenářského plánu
+• Jak si vybrat knihu: práce s anotací, obálkou, prvními stránkami; pravidlo „5 stran“ a odvaha knihu odložit
+• Čtenářské strategie v praxi: předvídání, vizualizace, propojování s vlastním životem, hlasité přemýšlení nad textem
+• Kniha, která mě něco naučila: hledání postav a situací podobných vlastnímu životu a co si z nich vzít
+• Čtenářský klub: doporučování knih spolužákům, diskuse nad přečteným, návštěva knihovny nebo autorské čtení</t>
+        </is>
+      </c>
+      <c r="I52" s="3" t="inlineStr">
+        <is>
+          <t>• metakognice čtení, kritické čtenářství
+• Český jazyk a literatura: čtenářské strategie, tvořivá práce s literárním textem, reflexe zážitku z četby
+• Osobnostní a sociální výchova: hledání vzorů a etických otázek v literatuře</t>
+        </is>
+      </c>
+      <c r="J52" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K52" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K51"/>
+  <autoFilter ref="A1:K52"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3814,17 +3874,17 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>13, 17, 49</t>
+          <t>13, 17, 49, 51</t>
         </is>
       </c>
       <c r="F3" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H3" s="3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4">
@@ -3881,7 +3941,7 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>17, 51</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -3890,13 +3950,13 @@
         </is>
       </c>
       <c r="F5" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G5" s="3" t="n">
         <v>2</v>
       </c>
       <c r="H5" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
@@ -4174,17 +4234,17 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>44, 48</t>
+          <t>44, 48, 51</t>
         </is>
       </c>
       <c r="F13" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H13" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="14">
@@ -4714,17 +4774,17 @@
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>7, 51</t>
         </is>
       </c>
       <c r="F28" s="3" t="n">
         <v>0</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H28" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="29">
@@ -6514,17 +6574,17 @@
       </c>
       <c r="E78" s="3" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>12, 51</t>
         </is>
       </c>
       <c r="F78" s="3" t="n">
         <v>0</v>
       </c>
       <c r="G78" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H78" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="79">

</xml_diff>

<commit_message>
Krev do tématu 9, IZS do tématu 36, nové téma 52 Bushcraft
Třetí dávka nápadů od kolegů:
- téma 9 Doktor v nás: nová aktivita „Krev pod lupou" (oběh, krevní skupiny,
  dárcovství krve a plazmy), transfuzní stanice doplněna do exkurzí,
  doplněny všechny tři diferenciace
- téma 36 Nouzový režim: nová aktivita o složkách IZS, návštěvě policejní
  stanice a aplikaci Záchranka; doplněny diferenciace
- nové téma 52 Bushcraft: doma v přírodě (SC8, vedoucí kameny 8.2.6.2
  a 4.2.1.4, dosud nevyužité) — dovednosti pobytu venku odděleně od tématu 7
  Expedice, které je o výpravě, ne o dovednostech
- podklady/odlozene_napady.md: zdůvodnění odložení tématu o letectví
  (kámen o principiálních poznatcích je v návrhu SC2 zatím bez umístění)

Katalog má nyní 52 témat, README aktualizováno, přegenerován web, Word i Excel.
</commit_message>
<xml_diff>
--- a/vystupy/Projektova_temata.xlsx
+++ b/vystupy/Projektova_temata.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Jak s tabulkou pracovat" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Témata'!$A$1:$K$52</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Témata'!$A$1:$K$53</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Pokrytí kamenů'!$A$1:$H$121</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -507,7 +507,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K52"/>
+  <dimension ref="A1:K53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1112,8 +1112,9 @@
           <t>• Cesta nemoci tělem: viry, bakterie, imunita — pokusy a modely (šíření „nákazy“ ve třídě jako simulace)
 • Domácí lékárnička: co v ní má být, k čemu léky slouží a jaká mají rizika
 • Simulace návštěvy lékaře: objednání, popis příznaků, porozumění diagnóze; orientace v systému (praktik, specialista, pohotovost, pojišťovna)
-• Exkurze do nemocnice, lékárny či záchranné stanice, beseda se zdravotníkem
-• Historie medicíny: od bylinek k antibiotikům a vakcínám, největší objevy</t>
+• Exkurze do nemocnice, lékárny, transfuzní stanice či záchranné stanice, beseda se zdravotníkem
+• Historie medicíny: od bylinek k antibiotikům a vakcínám, největší objevy
+• Krev pod lupou: krevní oběh a srdce, složení krve, krevní skupiny a příběh jejich objevu; dárcovství krve a plazmy — proč lidé darují a komu to pomůže</t>
         </is>
       </c>
       <c r="I10" s="3" t="inlineStr">
@@ -1122,7 +1123,8 @@
 • Přírodopis: biologie člověka — orgánové soustavy, viry a bakterie, nemoci a prevence
 • Chemie: léčiva a návykové látky; bezpečná práce s látkami
 • Výchova ke zdraví a bezpečí: ochrana a podpora zdraví, prevence přenosných chorob
-• Dějepis: dějiny medicíny — od morových ran k vakcínám</t>
+• Dějepis: dějiny medicíny — od morových ran k vakcínám
+• Přírodopis: oběhová soustava — srdce, cévy, složení krve; krevní skupiny a transfuze</t>
         </is>
       </c>
       <c r="J10" s="3" t="inlineStr">
@@ -2792,7 +2794,8 @@
 • Evakuační cvičení naostro: plán, sraz, nouzové zavazadlo (co si vzít za 5 minut)
 • Přežití v přírodě: orientace bez mobilu, oheň, přístřešek, úprava vody, signalizace
 • Exkurze k hasičům či na krizové řízení města, beseda se záchranářem
-• Simulované krize v týmech: blackout, ztracený člen, zranění na výletě — jednání podle postupu Zastav se–Zhodnoť–Naplánuj–Jednej</t>
+• Simulované krize v týmech: blackout, ztracený člen, zranění na výletě — jednání podle postupu Zastav se–Zhodnoť–Naplánuj–Jednej
+• Kdo mi přijede na pomoc: složky integrovaného záchranného systému (hasiči, policie, zdravotnická záchranná služba) a kdo řeší co; návštěva policejní stanice, aplikace Záchranka v mobilu</t>
         </is>
       </c>
       <c r="I37" s="3" t="inlineStr">
@@ -2801,7 +2804,8 @@
 • Výchova ke zdraví a bezpečí: osobní bezpečí za mimořádných událostí a obrana státu (v revizi posílený okruh!); bezpečnost v dopravě
 • Geografie: živelní pohromy, chování při ohrožení, orientace v terénu
 • Fyzika: energie a její zdroje (blackout); Chemie: hořlaviny a nebezpečné látky
-• Tělesná výchova: pobyt a přežití v přírodě</t>
+• Tělesná výchova: pobyt a přežití v přírodě
+• Výchova k občanství: integrovaný záchranný systém — složky, jejich úkoly a spolupráce</t>
         </is>
       </c>
       <c r="J37" s="3" t="inlineStr">
@@ -3748,8 +3752,72 @@
       </c>
       <c r="K52" s="3" t="inlineStr"/>
     </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>Bushcraft: doma v přírodě</t>
+        </is>
+      </c>
+      <c r="C53" s="7" t="inlineStr">
+        <is>
+          <t>SC8 Mám život ve svých rukou</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>8.2.6.2 Zmírňuji či akceptuji rizika
+4.2.1.4 Chystám se na budoucí zátěžové situace</t>
+        </is>
+      </c>
+      <c r="E53" s="3" t="inlineStr">
+        <is>
+          <t>8.2.5.1 Zacházím se stroji a nástroji
+8.2.3.1 Postarám se o stravování
+4.1.1.6 Odpočívám
+8.2.3.4 Dopravuji se
+1.1.2.6 Učím se činností</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>1.–3.</t>
+        </is>
+      </c>
+      <c r="G53" s="3" t="inlineStr">
+        <is>
+          <t>Umět si venku poradit není jedna výprava, ale sada dovedností, které se dají trénovat celý rok za školou. Projekt učí být v přírodě soběstačný: rozdělat oheň i za mokra, uvázat správný uzel, postavit přístřešek, sbalit batoh, uvařit na ohni a obléknout se tak, aby zima ani déšť nebyly problém. Na rozdíl od Expedice tu nejde o cestu, ale o dovednosti samotné — a o vědomé zmírňování rizik, která s pobytem venku přicházejí.</t>
+        </is>
+      </c>
+      <c r="H53" s="3" t="inlineStr">
+        <is>
+          <t>• Oheň a vaření venku: rozdělání ohně různými způsoby a v různém počasí, bezpečnost ohniště, vaření v kotlíku a specifika venkovní kuchyně
+• Uzly a přístřešek: základní uzly a jejich použití, stavba přístřešku z plachty i přírodního materiálu, spaní venku nanečisto
+• Batoh a výstroj: co si vzít a co nechat doma, vrstvení oblečení pro zimu i léto, péče o nůž a nástroje
+• Terén a počasí: pohyb po sněhu a ledu, čtení počasí, orientace bez mobilu, co dělat, když se ochladí nebo začne pršet
+• Zkouška dovednosti: tábornický okruh stanovišť v různých ročních obdobích — každý ukáže, co už zvládne sám</t>
+        </is>
+      </c>
+      <c r="I53" s="3" t="inlineStr">
+        <is>
+          <t>• principy přežití v přírodě, plán B
+• Tělesná výchova: turistika a pobyt v přírodě, bezpečnost při pohybových aktivitách
+• Polytechnická výchova a praktické činnosti: bezpečná práce s nářadím (nůž, pila), příprava pokrmů v improvizovaných podmínkách
+• Fyzika: teplo a hoření, vedení tepla (vrstvení oblečení)
+• Výchova ke zdraví a bezpečí: prevence úrazů, podchlazení a přehřátí, chování při ohrožení</t>
+        </is>
+      </c>
+      <c r="J53" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K53" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K52"/>
+  <autoFilter ref="A1:K53"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4126,17 +4194,17 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>15, 38, 48</t>
+          <t>15, 38, 48, 52</t>
         </is>
       </c>
       <c r="F10" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="11">
@@ -4990,17 +5058,17 @@
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>3, 4, 5</t>
+          <t>3, 4, 5, 52</t>
         </is>
       </c>
       <c r="F34" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H34" s="3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="35">
@@ -5201,7 +5269,7 @@
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>52</t>
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr">
@@ -5210,13 +5278,13 @@
         </is>
       </c>
       <c r="F40" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G40" s="3" t="n">
         <v>1</v>
       </c>
       <c r="H40" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="41">
@@ -7330,17 +7398,17 @@
       </c>
       <c r="E99" s="3" t="inlineStr">
         <is>
-          <t>2, 39</t>
+          <t>2, 39, 52</t>
         </is>
       </c>
       <c r="F99" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G99" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H99" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="100">
@@ -7438,17 +7506,17 @@
       </c>
       <c r="E102" s="3" t="inlineStr">
         <is>
-          <t>7, 19, 27, 29, 36</t>
+          <t>7, 19, 27, 29, 36, 52</t>
         </is>
       </c>
       <c r="F102" s="3" t="n">
         <v>0</v>
       </c>
       <c r="G102" s="3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H102" s="3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="103">
@@ -7546,17 +7614,17 @@
       </c>
       <c r="E105" s="3" t="inlineStr">
         <is>
-          <t>18, 46</t>
+          <t>18, 46, 52</t>
         </is>
       </c>
       <c r="F105" s="3" t="n">
         <v>2</v>
       </c>
       <c r="G105" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H105" s="3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="106">
@@ -7685,7 +7753,7 @@
       </c>
       <c r="D109" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>52</t>
         </is>
       </c>
       <c r="E109" s="3" t="inlineStr">
@@ -7694,13 +7762,13 @@
         </is>
       </c>
       <c r="F109" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G109" s="3" t="n">
         <v>2</v>
       </c>
       <c r="H109" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="110">

</xml_diff>

<commit_message>
Nové téma 53 Když slova nestačí (SC5, alternativní komunikace)
Podle návrhu kolegy na projekt o alternativní komunikaci. Vedoucí kámen
5.3.1.2 Domlouvám se s jinými — piktogramové tabulky a systémy AAC, znak
do řeči a znakový jazyk, Braillovo písmo, komunikační aplikace, setkání
s člověkem, který alternativní komunikaci používá.

Fyzikální část návrhu nová témata nevyžaduje — pokrývají ji už témata 47
(Elektřina), 48 (Světlo a zvuk) a 49 (Vesmír).

Katalog má nyní 53 témat, README aktualizováno, přegenerován web, Word i Excel.
</commit_message>
<xml_diff>
--- a/vystupy/Projektova_temata.xlsx
+++ b/vystupy/Projektova_temata.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Jak s tabulkou pracovat" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Témata'!$A$1:$K$53</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Témata'!$A$1:$K$54</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Pokrytí kamenů'!$A$1:$H$121</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -507,7 +507,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K53"/>
+  <dimension ref="A1:K54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3816,8 +3816,71 @@
       </c>
       <c r="K53" s="3" t="inlineStr"/>
     </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>Když slova nestačí</t>
+        </is>
+      </c>
+      <c r="C54" s="6" t="inlineStr">
+        <is>
+          <t>SC5 Buduji dobré vztahy</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="inlineStr">
+        <is>
+          <t>5.3.1.2 Domlouvám se s jinými</t>
+        </is>
+      </c>
+      <c r="E54" s="3" t="inlineStr">
+        <is>
+          <t>5.1.1.1 Vnímám a přijímám druhé
+5.3.2.1 Komunikuji s respektem
+1.1.2.4 Získávám poznatky z nejazykových druhů vyjádření
+5.3.1.4 Ovládám komunikační kanály
+8.2.4.1 Využívám digitální technologie</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>1.–3.</t>
+        </is>
+      </c>
+      <c r="G54" s="3" t="inlineStr">
+        <is>
+          <t>Co když člověk nemůže mluvit — nebo mluví jiným jazykem než ty? Projekt o komunikaci, která si musí poradit bez běžné řeči: piktogramové tabulky a komunikační knihy, znak do řeči a znakový jazyk, Braillovo písmo, gesta a mimika i komunikační aplikace na tabletu. Děti si na vlastní kůži zkusí, jaké to je nemoci říct, co potřebuji — a naučí se, jak se dá dorozumět, když slova nestačí.</t>
+        </is>
+      </c>
+      <c r="H54" s="3" t="inlineStr">
+        <is>
+          <t>• Hodina beze slov: domluvit se na společném úkolu bez mluvené řeči (gesta, kresba, piktogramy) a pojmenovat, co bylo nejtěžší
+• Piktogramy a komunikační tabulky: jak fungují systémy alternativní komunikace, výroba vlastní tabulky či knihy pro konkrétní situaci (jídelna, výlet)
+• Znakový jazyk a znak do řeči: základy od lektora či neslyšícího hosta — pozdrav, představení se, běžné fráze; proč je znakový jazyk plnohodnotný jazyk, ne pantomima
+• Braille a další jazyky beze slov: hmatové písmo, morseovka, mezinárodní symboly — vyzkoušení a porovnání, čím se který hodí
+• Setkání naostro: návštěva organizace pracující s lidmi s postižením komunikace nebo host ve škole; rozhovor připravený tak, aby se domluvily obě strany</t>
+        </is>
+      </c>
+      <c r="I54" s="3" t="inlineStr">
+        <is>
+          <t>• Výchova ke zdraví a bezpečí: vztahy mezi lidmi, respekt k odlišnosti, soužití s lidmi se znevýhodněním
+• Český jazyk a literatura: komunikační situace a záměr, aktivní naslouchání, neverbální komunikace
+• Informatika: kódování informace (Braillovo písmo, morseovka), asistivní technologie a komunikační aplikace
+• Osobnostní a sociální výchova: empatie, přijímání odlišnosti, komunikace v náročných situacích
+• Výtvarná a filmová výchova: piktogram a vizuální znak jako nositel významu</t>
+        </is>
+      </c>
+      <c r="J54" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K54" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K53"/>
+  <autoFilter ref="A1:K54"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4122,17 +4185,17 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>17, 48, 49</t>
+          <t>17, 48, 49, 53</t>
         </is>
       </c>
       <c r="F8" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9">
@@ -5598,17 +5661,17 @@
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>24, 27, 42</t>
+          <t>24, 27, 42, 53</t>
         </is>
       </c>
       <c r="F49" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G49" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H49" s="3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="50">
@@ -6601,7 +6664,7 @@
       </c>
       <c r="D77" s="3" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>21, 53</t>
         </is>
       </c>
       <c r="E77" s="3" t="inlineStr">
@@ -6610,13 +6673,13 @@
         </is>
       </c>
       <c r="F77" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G77" s="3" t="n">
         <v>3</v>
       </c>
       <c r="H77" s="3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="78">
@@ -6678,17 +6741,17 @@
       </c>
       <c r="E79" s="3" t="inlineStr">
         <is>
-          <t>28, 30</t>
+          <t>28, 30, 53</t>
         </is>
       </c>
       <c r="F79" s="3" t="n">
         <v>0</v>
       </c>
       <c r="G79" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H79" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="80">
@@ -6714,17 +6777,17 @@
       </c>
       <c r="E80" s="3" t="inlineStr">
         <is>
-          <t>6, 22</t>
+          <t>6, 22, 53</t>
         </is>
       </c>
       <c r="F80" s="3" t="n">
         <v>0</v>
       </c>
       <c r="G80" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H80" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="81">
@@ -7542,17 +7605,17 @@
       </c>
       <c r="E103" s="3" t="inlineStr">
         <is>
-          <t>12, 47</t>
+          <t>12, 47, 53</t>
         </is>
       </c>
       <c r="F103" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G103" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H103" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="104">

</xml_diff>

<commit_message>
Téma 43: poznámka o volbách patří do anotace, ne mezi aktivity
„Mimořádné zařazení podle kalendáře" nebyla aktivita, ale informace
o tématu, a dělala z tématu 43 jediné se sedmi aktivitami v katalogu.
Přesunuto na konec anotace — informace zůstává průvodci na očích a rozsah
aktivit je zpět na 5–6 u všech 55 témat.

Přegenerován web, Word i Excel.
</commit_message>
<xml_diff>
--- a/vystupy/Projektova_temata.xlsx
+++ b/vystupy/Projektova_temata.xlsx
@@ -3250,7 +3250,7 @@
       </c>
       <c r="G44" s="3" t="inlineStr">
         <is>
-          <t>Kdo rozhoduje o tom, co smím a co musím — a jak to můžu ovlivnit? Projekt rozebírá stát od obce po mezinárodní instituce: volby, parlament, vláda a soudy, obecní zastupitelstvo, EU, NATO i OSN. Děti si stát vyzkoušejí zevnitř — simulací voleb a parlamentu — a naostro navštíví úřady a zastupitele.</t>
+          <t>Kdo rozhoduje o tom, co smím a co musím — a jak to můžu ovlivnit? Projekt rozebírá stát od obce po mezinárodní instituce: volby, parlament, vláda a soudy, obecní zastupitelstvo, EU, NATO i OSN. Děti si stát vyzkoušejí zevnitř — simulací voleb a parlamentu — a naostro navštíví úřady a zastupitele. Konají-li se právě skutečné volby (prezidentské, parlamentní i komunální), vyplatí se téma zařadit i mimo plánovaný blok — děti ho pak zažijí v reálném čase.</t>
         </is>
       </c>
       <c r="H44" s="3" t="inlineStr">
@@ -3260,8 +3260,7 @@
 • Návštěva jednání obecního zastupitelstva, radnice či Poslanecké sněmovny; rozhovor se zastupitelem
 • Mapa institucí: kdo mi vydá občanku, kdo opravuje silnici, kdo mě soudí, co dělá EU/NATO/OSN — a kam se obrátit se skutečným podnětem
 • Občanský projekt naostro: podnět či petice k reálnému problému v okolí školy (přechod, hřiště, koš)
-• Vlajka, znak a hymna: co znamenají státní symboly a proč je máme; procházka obcí za pamětihodnostmi jako symboly domova
-• Mimořádné zařazení podle kalendáře: konají-li se skutečné volby (prezidentské, parlamentní, komunální), lze projekt zařadit i mimo plánovaný blok, aby ho děti zažily v reálném čase</t>
+• Vlajka, znak a hymna: co znamenají státní symboly a proč je máme; procházka obcí za pamětihodnostmi jako symboly domova</t>
         </is>
       </c>
       <c r="I44" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Odebrat téma 52 Bushcraft
Úzce zaměřené — spíš samostatný předmět než široké téma, které si průvodce
postaví po svém. Dovednosti pobytu venku zůstávají v tématu 7 Expedice
a 36 Nouzový režim.

Kameny 8.2.6.2 Zmírňuji či akceptuji rizika a 4.2.1.4 Chystám se na budoucí
zátěžové situace tím ztrácejí vedoucí téma, zůstávají ale vedlejší u tématu 36
(8.2.6.2 navíc u 47), takže žádný kámen nezůstal nepokrytý — jediný nepokrytý
je i nadále záměrný 5.2.3.3.

Katalog má 54 témat. Id 52 se neuvolňuje pro další použití; poznámky doplněny
o toto rozhodnutí i o pravidlo, že se id nepřečíslovávají.

Přegenerován web, Word i Excel.
</commit_message>
<xml_diff>
--- a/vystupy/Projektova_temata.xlsx
+++ b/vystupy/Projektova_temata.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Jak s tabulkou pracovat" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Témata'!$A$1:$K$56</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Témata'!$A$1:$K$55</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Pokrytí kamenů'!$A$1:$H$121</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -507,7 +507,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K56"/>
+  <dimension ref="A1:K55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3782,89 +3782,24 @@
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>Bushcraft: doma v přírodě</t>
-        </is>
-      </c>
-      <c r="C53" s="7" t="inlineStr">
-        <is>
-          <t>SC8 Mám život ve svých rukou</t>
+          <t>Když slova nestačí</t>
+        </is>
+      </c>
+      <c r="C53" s="6" t="inlineStr">
+        <is>
+          <t>SC5 Buduji dobré vztahy</t>
         </is>
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>8.2.6.2 Zmírňuji či akceptuji rizika
-4.2.1.4 Chystám se na budoucí zátěžové situace</t>
+          <t>5.3.1.2 Domlouvám se s jinými</t>
         </is>
       </c>
       <c r="E53" s="3" t="inlineStr">
-        <is>
-          <t>8.2.5.1 Zacházím se stroji a nástroji
-8.2.3.1 Postarám se o stravování
-4.1.1.6 Odpočívám
-8.2.3.4 Dopravuji se
-1.1.2.6 Učím se činností</t>
-        </is>
-      </c>
-      <c r="F53" s="2" t="inlineStr">
-        <is>
-          <t>1.–3.</t>
-        </is>
-      </c>
-      <c r="G53" s="3" t="inlineStr">
-        <is>
-          <t>Umět si venku poradit není jedna výprava, ale sada dovedností, které se dají trénovat celý rok za školou. Projekt učí být v přírodě soběstačný: rozdělat oheň i za mokra, uvázat správný uzel, postavit přístřešek, sbalit batoh, uvařit na ohni a obléknout se tak, aby zima ani déšť nebyly problém. Na rozdíl od Expedice tu nejde o cestu, ale o dovednosti samotné — a o vědomé zmírňování rizik, která s pobytem venku přicházejí.</t>
-        </is>
-      </c>
-      <c r="H53" s="3" t="inlineStr">
-        <is>
-          <t>• Oheň a vaření venku: rozdělání ohně různými způsoby a v různém počasí, bezpečnost ohniště, vaření v kotlíku a specifika venkovní kuchyně
-• Uzly a přístřešek: základní uzly a jejich použití, stavba přístřešku z plachty i přírodního materiálu, spaní venku nanečisto
-• Batoh a výstroj: co si vzít a co nechat doma, vrstvení oblečení pro zimu i léto, péče o nůž a nástroje
-• Terén a počasí: pohyb po sněhu a ledu, čtení počasí, orientace bez mobilu, co dělat, když se ochladí nebo začne pršet
-• Zkouška dovednosti: tábornický okruh stanovišť v různých ročních obdobích — každý ukáže, co už zvládne sám</t>
-        </is>
-      </c>
-      <c r="I53" s="3" t="inlineStr">
-        <is>
-          <t>• principy přežití v přírodě, plán B
-• Tělesná výchova: turistika a pobyt v přírodě, bezpečnost při pohybových aktivitách
-• Polytechnická výchova a praktické činnosti: bezpečná práce s nářadím (nůž, pila), příprava pokrmů v improvizovaných podmínkách
-• Fyzika: teplo a hoření, vedení tepla (vrstvení oblečení)
-• Výchova ke zdraví a bezpečí: prevence úrazů, podchlazení a přehřátí, chování při ohrožení
-• Přírodopis: horniny, nerosty a tvary krajiny v terénu; orientace podle přírodních znaků</t>
-        </is>
-      </c>
-      <c r="J53" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K53" s="3" t="inlineStr"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="2" t="n">
-        <v>53</v>
-      </c>
-      <c r="B54" s="3" t="inlineStr">
-        <is>
-          <t>Když slova nestačí</t>
-        </is>
-      </c>
-      <c r="C54" s="6" t="inlineStr">
-        <is>
-          <t>SC5 Buduji dobré vztahy</t>
-        </is>
-      </c>
-      <c r="D54" s="3" t="inlineStr">
-        <is>
-          <t>5.3.1.2 Domlouvám se s jinými</t>
-        </is>
-      </c>
-      <c r="E54" s="3" t="inlineStr">
         <is>
           <t>5.1.1.1 Vnímám a přijímám druhé
 5.3.2.1 Komunikuji s respektem
@@ -3873,17 +3808,17 @@
 8.2.4.1 Využívám digitální technologie</t>
         </is>
       </c>
-      <c r="F54" s="2" t="inlineStr">
+      <c r="F53" s="2" t="inlineStr">
         <is>
           <t>1.–3.</t>
         </is>
       </c>
-      <c r="G54" s="3" t="inlineStr">
+      <c r="G53" s="3" t="inlineStr">
         <is>
           <t>Co když člověk nemůže mluvit — nebo mluví jiným jazykem než ty? Projekt o komunikaci, která si musí poradit bez běžné řeči: piktogramové tabulky a komunikační knihy, znak do řeči a znakový jazyk, Braillovo písmo, gesta a mimika i komunikační aplikace na tabletu. Děti si na vlastní kůži zkusí, jaké to je nemoci říct, co potřebuji — a naučí se, jak se dá dorozumět, když slova nestačí.</t>
         </is>
       </c>
-      <c r="H54" s="3" t="inlineStr">
+      <c r="H53" s="3" t="inlineStr">
         <is>
           <t>• Hodina beze slov: domluvit se na společném úkolu bez mluvené řeči (gesta, kresba, piktogramy) a pojmenovat, co bylo nejtěžší
 • Piktogramy a komunikační tabulky: jak fungují systémy alternativní komunikace, výroba vlastní tabulky či knihy pro konkrétní situaci (jídelna, výlet)
@@ -3892,7 +3827,7 @@
 • Setkání naostro: návštěva organizace pracující s lidmi s postižením komunikace nebo host ve škole; rozhovor připravený tak, aby se domluvily obě strany</t>
         </is>
       </c>
-      <c r="I54" s="3" t="inlineStr">
+      <c r="I53" s="3" t="inlineStr">
         <is>
           <t>• Výchova ke zdraví a bezpečí: vztahy mezi lidmi, respekt k odlišnosti, soužití s lidmi se znevýhodněním
 • Český jazyk a literatura: komunikační situace a záměr, aktivní naslouchání, neverbální komunikace
@@ -3901,35 +3836,35 @@
 • Výtvarná a filmová výchova: piktogram a vizuální znak jako nositel významu</t>
         </is>
       </c>
-      <c r="J54" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K54" s="3" t="inlineStr"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="2" t="n">
+      <c r="J53" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K53" s="3" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
         <v>54</v>
       </c>
-      <c r="B55" s="3" t="inlineStr">
+      <c r="B54" s="3" t="inlineStr">
         <is>
           <t>Zvládnu to sám!</t>
         </is>
       </c>
-      <c r="C55" s="4" t="inlineStr">
+      <c r="C54" s="4" t="inlineStr">
         <is>
           <t>SC4 Rozvíjím svou odolnost</t>
         </is>
       </c>
-      <c r="D55" s="3" t="inlineStr">
+      <c r="D54" s="3" t="inlineStr">
         <is>
           <t>4.2.1.1 Jsem připraven/a na výzvy
 8.2.3.4 Dopravuji se
 5.1.1.6 Hlídám si hranice</t>
         </is>
       </c>
-      <c r="E55" s="3" t="inlineStr">
+      <c r="E54" s="3" t="inlineStr">
         <is>
           <t>4.2.2.4 Sdílím a říkám si o pomoc
 5.1.2.2 Navazuji kontakty
@@ -3938,17 +3873,17 @@
 8.2.3.3 Obstarávám si věci a zařizuji služby</t>
         </is>
       </c>
-      <c r="F55" s="2" t="inlineStr">
+      <c r="F54" s="2" t="inlineStr">
         <is>
           <t>jen 1.</t>
         </is>
       </c>
-      <c r="G55" s="3" t="inlineStr">
+      <c r="G54" s="3" t="inlineStr">
         <is>
           <t>Být poprvé v něčem sám je malé dobrodružství — a dá se na něj připravit. Projekt je sbírkou prvních samostatných činů šitých na míru nejmenším: dojít známou cestou bez dospělého, koupit rohlík, půjčit si knihu, oslovit cizího člověka a zeptat se na cestu. Ke každé odvaze patří i druhá strana samostatnosti: umět říct „ne“, poznat tíživé tajemství a vědět, komu se svěřím. Děti sbírají odznaky do vlastního Průkazu samostatnosti — každý za něco, co teď už zvládnou samy.</t>
         </is>
       </c>
-      <c r="H55" s="3" t="inlineStr">
+      <c r="H54" s="3" t="inlineStr">
         <is>
           <t>• Průkaz samostatnosti: společně vymyslet, co všechno chceme letos zvládnout sami; každý si vybere své výzvy a odškrtává splněné odznaky
 • Cesta, kterou znám: okolí školy, dopravní značky a pravidla pro chodce, samostatná cesta na známé místo (knihovna, park, obchod) s průvodcem jistícím z pozadí
@@ -3957,7 +3892,7 @@
 • Slavnost odznaků: každý předvede, co už zvládne sám, a ukáže to mladším dětem nebo rodičům</t>
         </is>
       </c>
-      <c r="I55" s="3" t="inlineStr">
+      <c r="I54" s="3" t="inlineStr">
         <is>
           <t>• Člověk a jeho svět: bezpečná cesta do školy, dopravní značky a pravidla pro chodce, osobní bezpečí, důležitá telefonní čísla
 • Výchova ke zdraví a bezpečí: osobní bezpečí, hranice a odmítání, kde hledat pomoc
@@ -3965,35 +3900,35 @@
 • Český jazyk a literatura: zdvořilostní obraty, oslovení a prosba o pomoc</t>
         </is>
       </c>
-      <c r="J55" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K55" s="3" t="inlineStr"/>
-    </row>
-    <row r="56">
-      <c r="A56" s="2" t="n">
+      <c r="J54" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K54" s="3" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
         <v>55</v>
       </c>
-      <c r="B56" s="3" t="inlineStr">
+      <c r="B55" s="3" t="inlineStr">
         <is>
           <t>Naše třída: jak si tu spolu žijeme</t>
         </is>
       </c>
-      <c r="C56" s="6" t="inlineStr">
+      <c r="C55" s="6" t="inlineStr">
         <is>
           <t>SC5 Buduji dobré vztahy</t>
         </is>
       </c>
-      <c r="D56" s="3" t="inlineStr">
+      <c r="D55" s="3" t="inlineStr">
         <is>
           <t>5.1.1.2 Někam patřím a přijímám ostatní
 5.1.1.5 Nakládám s hranicemi a autoritou
 5.3.2.1 Komunikuji s respektem</t>
         </is>
       </c>
-      <c r="E56" s="3" t="inlineStr">
+      <c r="E55" s="3" t="inlineStr">
         <is>
           <t>5.1.1.10 Poskytuji a přijímám zpětnou vazbu
 5.1.1.8 Nakládám s autoritou
@@ -4002,17 +3937,17 @@
 1.2.4.2 Reflektuji průběh cíleného učení</t>
         </is>
       </c>
-      <c r="F56" s="2" t="inlineStr">
+      <c r="F55" s="2" t="inlineStr">
         <is>
           <t>jen 1.</t>
         </is>
       </c>
-      <c r="G56" s="3" t="inlineStr">
+      <c r="G55" s="3" t="inlineStr">
         <is>
           <t>Třída není daná, dělá se. Projekt bere soužití ve třídě jako věc, kterou děti samy tvoří: společně vyvodí pravidla a zjistí, proč vlastně jsou, rozdělí si služby a vyzkoušejí různé role ve skupině, všímají si, kdo zůstává stranou, a učí se říct druhému, co mu jde. Na konci třída ví, co jí funguje a co chce jinak — a má to černé na bílém.</t>
         </is>
       </c>
-      <c r="H56" s="3" t="inlineStr">
+      <c r="H55" s="3" t="inlineStr">
         <is>
           <t>• Třídní ústava: společné vyvození pravidel — proč je máme a co se stane, když je někdo poruší; vyvěšení, podpis a revize na konci projektu
 • Služby a role: kdo se u nás o co stará (rostlina, knihovnička, kruh) a vyzkoušení různých rolí ve skupinové práci — i té, která mi nesedí
@@ -4021,7 +3956,7 @@
 • Kruh ocenění: co komu jde a čím nám pomáhá; nácvik konkrétní pochvaly i věcného postřehu; závěrečné „co nám tu funguje a co chceme jinak“</t>
         </is>
       </c>
-      <c r="I56" s="3" t="inlineStr">
+      <c r="I55" s="3" t="inlineStr">
         <is>
           <t>• Člověk a jeho svět: vztahy v rodině, ve třídě a ve škole; pravidla soužití a jejich vyvozování; tolerance k odlišnostem
 • Osobnostní a sociální výchova: sebepoznání a poznávání druhých, mezilidské vztahy, spolupráce a role ve skupině
@@ -4029,15 +3964,15 @@
 • Český jazyk a literatura: pravidla dialogu, střídání se v hovoru, formulace ocenění a věcného postřehu</t>
         </is>
       </c>
-      <c r="J56" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K56" s="3" t="inlineStr"/>
+      <c r="J55" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K55" s="3" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K56"/>
+  <autoFilter ref="A1:K55"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4414,17 +4349,17 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>15, 38, 48, 52</t>
+          <t>15, 38, 48</t>
         </is>
       </c>
       <c r="F10" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G10" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="H10" s="3" t="n">
         <v>4</v>
-      </c>
-      <c r="H10" s="3" t="n">
-        <v>5</v>
       </c>
     </row>
     <row r="11">
@@ -5278,17 +5213,17 @@
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>3, 4, 5, 52</t>
+          <t>3, 4, 5</t>
         </is>
       </c>
       <c r="F34" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G34" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="H34" s="3" t="n">
         <v>4</v>
-      </c>
-      <c r="H34" s="3" t="n">
-        <v>5</v>
       </c>
     </row>
     <row r="35">
@@ -5489,7 +5424,7 @@
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>52</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr">
@@ -5498,13 +5433,13 @@
         </is>
       </c>
       <c r="F40" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G40" s="3" t="n">
         <v>1</v>
       </c>
       <c r="H40" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="41">
@@ -7618,17 +7553,17 @@
       </c>
       <c r="E99" s="3" t="inlineStr">
         <is>
-          <t>2, 39, 52</t>
+          <t>2, 39</t>
         </is>
       </c>
       <c r="F99" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G99" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="H99" s="3" t="n">
         <v>3</v>
-      </c>
-      <c r="H99" s="3" t="n">
-        <v>4</v>
       </c>
     </row>
     <row r="100">
@@ -7726,17 +7661,17 @@
       </c>
       <c r="E102" s="3" t="inlineStr">
         <is>
-          <t>7, 19, 27, 29, 36, 52</t>
+          <t>7, 19, 27, 29, 36</t>
         </is>
       </c>
       <c r="F102" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G102" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="H102" s="3" t="n">
         <v>6</v>
-      </c>
-      <c r="H102" s="3" t="n">
-        <v>7</v>
       </c>
     </row>
     <row r="103">
@@ -7834,17 +7769,17 @@
       </c>
       <c r="E105" s="3" t="inlineStr">
         <is>
-          <t>18, 46, 52</t>
+          <t>18, 46</t>
         </is>
       </c>
       <c r="F105" s="3" t="n">
         <v>2</v>
       </c>
       <c r="G105" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H105" s="3" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="106">
@@ -7973,7 +7908,7 @@
       </c>
       <c r="D109" s="3" t="inlineStr">
         <is>
-          <t>52</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E109" s="3" t="inlineStr">
@@ -7982,13 +7917,13 @@
         </is>
       </c>
       <c r="F109" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G109" s="3" t="n">
         <v>2</v>
       </c>
       <c r="H109" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="110">

</xml_diff>

<commit_message>
Revert "Odebrat téma 52 Bushcraft"
This reverts commit ddf75612590b3db79b7ffe2a408acdc69ffd7b0f.
</commit_message>
<xml_diff>
--- a/vystupy/Projektova_temata.xlsx
+++ b/vystupy/Projektova_temata.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Jak s tabulkou pracovat" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Témata'!$A$1:$K$55</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Témata'!$A$1:$K$56</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Pokrytí kamenů'!$A$1:$H$121</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -507,7 +507,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K55"/>
+  <dimension ref="A1:K56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3782,24 +3782,89 @@
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>Bushcraft: doma v přírodě</t>
+        </is>
+      </c>
+      <c r="C53" s="7" t="inlineStr">
+        <is>
+          <t>SC8 Mám život ve svých rukou</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>8.2.6.2 Zmírňuji či akceptuji rizika
+4.2.1.4 Chystám se na budoucí zátěžové situace</t>
+        </is>
+      </c>
+      <c r="E53" s="3" t="inlineStr">
+        <is>
+          <t>8.2.5.1 Zacházím se stroji a nástroji
+8.2.3.1 Postarám se o stravování
+4.1.1.6 Odpočívám
+8.2.3.4 Dopravuji se
+1.1.2.6 Učím se činností</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>1.–3.</t>
+        </is>
+      </c>
+      <c r="G53" s="3" t="inlineStr">
+        <is>
+          <t>Umět si venku poradit není jedna výprava, ale sada dovedností, které se dají trénovat celý rok za školou. Projekt učí být v přírodě soběstačný: rozdělat oheň i za mokra, uvázat správný uzel, postavit přístřešek, sbalit batoh, uvařit na ohni a obléknout se tak, aby zima ani déšť nebyly problém. Na rozdíl od Expedice tu nejde o cestu, ale o dovednosti samotné — a o vědomé zmírňování rizik, která s pobytem venku přicházejí.</t>
+        </is>
+      </c>
+      <c r="H53" s="3" t="inlineStr">
+        <is>
+          <t>• Oheň a vaření venku: rozdělání ohně různými způsoby a v různém počasí, bezpečnost ohniště, vaření v kotlíku a specifika venkovní kuchyně
+• Uzly a přístřešek: základní uzly a jejich použití, stavba přístřešku z plachty i přírodního materiálu, spaní venku nanečisto
+• Batoh a výstroj: co si vzít a co nechat doma, vrstvení oblečení pro zimu i léto, péče o nůž a nástroje
+• Terén a počasí: pohyb po sněhu a ledu, čtení počasí, orientace bez mobilu, co dělat, když se ochladí nebo začne pršet
+• Zkouška dovednosti: tábornický okruh stanovišť v různých ročních obdobích — každý ukáže, co už zvládne sám</t>
+        </is>
+      </c>
+      <c r="I53" s="3" t="inlineStr">
+        <is>
+          <t>• principy přežití v přírodě, plán B
+• Tělesná výchova: turistika a pobyt v přírodě, bezpečnost při pohybových aktivitách
+• Polytechnická výchova a praktické činnosti: bezpečná práce s nářadím (nůž, pila), příprava pokrmů v improvizovaných podmínkách
+• Fyzika: teplo a hoření, vedení tepla (vrstvení oblečení)
+• Výchova ke zdraví a bezpečí: prevence úrazů, podchlazení a přehřátí, chování při ohrožení
+• Přírodopis: horniny, nerosty a tvary krajiny v terénu; orientace podle přírodních znaků</t>
+        </is>
+      </c>
+      <c r="J53" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K53" s="3" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
         <v>53</v>
       </c>
-      <c r="B53" s="3" t="inlineStr">
+      <c r="B54" s="3" t="inlineStr">
         <is>
           <t>Když slova nestačí</t>
         </is>
       </c>
-      <c r="C53" s="6" t="inlineStr">
+      <c r="C54" s="6" t="inlineStr">
         <is>
           <t>SC5 Buduji dobré vztahy</t>
         </is>
       </c>
-      <c r="D53" s="3" t="inlineStr">
+      <c r="D54" s="3" t="inlineStr">
         <is>
           <t>5.3.1.2 Domlouvám se s jinými</t>
         </is>
       </c>
-      <c r="E53" s="3" t="inlineStr">
+      <c r="E54" s="3" t="inlineStr">
         <is>
           <t>5.1.1.1 Vnímám a přijímám druhé
 5.3.2.1 Komunikuji s respektem
@@ -3808,17 +3873,17 @@
 8.2.4.1 Využívám digitální technologie</t>
         </is>
       </c>
-      <c r="F53" s="2" t="inlineStr">
+      <c r="F54" s="2" t="inlineStr">
         <is>
           <t>1.–3.</t>
         </is>
       </c>
-      <c r="G53" s="3" t="inlineStr">
+      <c r="G54" s="3" t="inlineStr">
         <is>
           <t>Co když člověk nemůže mluvit — nebo mluví jiným jazykem než ty? Projekt o komunikaci, která si musí poradit bez běžné řeči: piktogramové tabulky a komunikační knihy, znak do řeči a znakový jazyk, Braillovo písmo, gesta a mimika i komunikační aplikace na tabletu. Děti si na vlastní kůži zkusí, jaké to je nemoci říct, co potřebuji — a naučí se, jak se dá dorozumět, když slova nestačí.</t>
         </is>
       </c>
-      <c r="H53" s="3" t="inlineStr">
+      <c r="H54" s="3" t="inlineStr">
         <is>
           <t>• Hodina beze slov: domluvit se na společném úkolu bez mluvené řeči (gesta, kresba, piktogramy) a pojmenovat, co bylo nejtěžší
 • Piktogramy a komunikační tabulky: jak fungují systémy alternativní komunikace, výroba vlastní tabulky či knihy pro konkrétní situaci (jídelna, výlet)
@@ -3827,7 +3892,7 @@
 • Setkání naostro: návštěva organizace pracující s lidmi s postižením komunikace nebo host ve škole; rozhovor připravený tak, aby se domluvily obě strany</t>
         </is>
       </c>
-      <c r="I53" s="3" t="inlineStr">
+      <c r="I54" s="3" t="inlineStr">
         <is>
           <t>• Výchova ke zdraví a bezpečí: vztahy mezi lidmi, respekt k odlišnosti, soužití s lidmi se znevýhodněním
 • Český jazyk a literatura: komunikační situace a záměr, aktivní naslouchání, neverbální komunikace
@@ -3836,35 +3901,35 @@
 • Výtvarná a filmová výchova: piktogram a vizuální znak jako nositel významu</t>
         </is>
       </c>
-      <c r="J53" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K53" s="3" t="inlineStr"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="2" t="n">
+      <c r="J54" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K54" s="3" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
         <v>54</v>
       </c>
-      <c r="B54" s="3" t="inlineStr">
+      <c r="B55" s="3" t="inlineStr">
         <is>
           <t>Zvládnu to sám!</t>
         </is>
       </c>
-      <c r="C54" s="4" t="inlineStr">
+      <c r="C55" s="4" t="inlineStr">
         <is>
           <t>SC4 Rozvíjím svou odolnost</t>
         </is>
       </c>
-      <c r="D54" s="3" t="inlineStr">
+      <c r="D55" s="3" t="inlineStr">
         <is>
           <t>4.2.1.1 Jsem připraven/a na výzvy
 8.2.3.4 Dopravuji se
 5.1.1.6 Hlídám si hranice</t>
         </is>
       </c>
-      <c r="E54" s="3" t="inlineStr">
+      <c r="E55" s="3" t="inlineStr">
         <is>
           <t>4.2.2.4 Sdílím a říkám si o pomoc
 5.1.2.2 Navazuji kontakty
@@ -3873,17 +3938,17 @@
 8.2.3.3 Obstarávám si věci a zařizuji služby</t>
         </is>
       </c>
-      <c r="F54" s="2" t="inlineStr">
+      <c r="F55" s="2" t="inlineStr">
         <is>
           <t>jen 1.</t>
         </is>
       </c>
-      <c r="G54" s="3" t="inlineStr">
+      <c r="G55" s="3" t="inlineStr">
         <is>
           <t>Být poprvé v něčem sám je malé dobrodružství — a dá se na něj připravit. Projekt je sbírkou prvních samostatných činů šitých na míru nejmenším: dojít známou cestou bez dospělého, koupit rohlík, půjčit si knihu, oslovit cizího člověka a zeptat se na cestu. Ke každé odvaze patří i druhá strana samostatnosti: umět říct „ne“, poznat tíživé tajemství a vědět, komu se svěřím. Děti sbírají odznaky do vlastního Průkazu samostatnosti — každý za něco, co teď už zvládnou samy.</t>
         </is>
       </c>
-      <c r="H54" s="3" t="inlineStr">
+      <c r="H55" s="3" t="inlineStr">
         <is>
           <t>• Průkaz samostatnosti: společně vymyslet, co všechno chceme letos zvládnout sami; každý si vybere své výzvy a odškrtává splněné odznaky
 • Cesta, kterou znám: okolí školy, dopravní značky a pravidla pro chodce, samostatná cesta na známé místo (knihovna, park, obchod) s průvodcem jistícím z pozadí
@@ -3892,7 +3957,7 @@
 • Slavnost odznaků: každý předvede, co už zvládne sám, a ukáže to mladším dětem nebo rodičům</t>
         </is>
       </c>
-      <c r="I54" s="3" t="inlineStr">
+      <c r="I55" s="3" t="inlineStr">
         <is>
           <t>• Člověk a jeho svět: bezpečná cesta do školy, dopravní značky a pravidla pro chodce, osobní bezpečí, důležitá telefonní čísla
 • Výchova ke zdraví a bezpečí: osobní bezpečí, hranice a odmítání, kde hledat pomoc
@@ -3900,35 +3965,35 @@
 • Český jazyk a literatura: zdvořilostní obraty, oslovení a prosba o pomoc</t>
         </is>
       </c>
-      <c r="J54" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K54" s="3" t="inlineStr"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="2" t="n">
+      <c r="J55" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K55" s="3" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
         <v>55</v>
       </c>
-      <c r="B55" s="3" t="inlineStr">
+      <c r="B56" s="3" t="inlineStr">
         <is>
           <t>Naše třída: jak si tu spolu žijeme</t>
         </is>
       </c>
-      <c r="C55" s="6" t="inlineStr">
+      <c r="C56" s="6" t="inlineStr">
         <is>
           <t>SC5 Buduji dobré vztahy</t>
         </is>
       </c>
-      <c r="D55" s="3" t="inlineStr">
+      <c r="D56" s="3" t="inlineStr">
         <is>
           <t>5.1.1.2 Někam patřím a přijímám ostatní
 5.1.1.5 Nakládám s hranicemi a autoritou
 5.3.2.1 Komunikuji s respektem</t>
         </is>
       </c>
-      <c r="E55" s="3" t="inlineStr">
+      <c r="E56" s="3" t="inlineStr">
         <is>
           <t>5.1.1.10 Poskytuji a přijímám zpětnou vazbu
 5.1.1.8 Nakládám s autoritou
@@ -3937,17 +4002,17 @@
 1.2.4.2 Reflektuji průběh cíleného učení</t>
         </is>
       </c>
-      <c r="F55" s="2" t="inlineStr">
+      <c r="F56" s="2" t="inlineStr">
         <is>
           <t>jen 1.</t>
         </is>
       </c>
-      <c r="G55" s="3" t="inlineStr">
+      <c r="G56" s="3" t="inlineStr">
         <is>
           <t>Třída není daná, dělá se. Projekt bere soužití ve třídě jako věc, kterou děti samy tvoří: společně vyvodí pravidla a zjistí, proč vlastně jsou, rozdělí si služby a vyzkoušejí různé role ve skupině, všímají si, kdo zůstává stranou, a učí se říct druhému, co mu jde. Na konci třída ví, co jí funguje a co chce jinak — a má to černé na bílém.</t>
         </is>
       </c>
-      <c r="H55" s="3" t="inlineStr">
+      <c r="H56" s="3" t="inlineStr">
         <is>
           <t>• Třídní ústava: společné vyvození pravidel — proč je máme a co se stane, když je někdo poruší; vyvěšení, podpis a revize na konci projektu
 • Služby a role: kdo se u nás o co stará (rostlina, knihovnička, kruh) a vyzkoušení různých rolí ve skupinové práci — i té, která mi nesedí
@@ -3956,7 +4021,7 @@
 • Kruh ocenění: co komu jde a čím nám pomáhá; nácvik konkrétní pochvaly i věcného postřehu; závěrečné „co nám tu funguje a co chceme jinak“</t>
         </is>
       </c>
-      <c r="I55" s="3" t="inlineStr">
+      <c r="I56" s="3" t="inlineStr">
         <is>
           <t>• Člověk a jeho svět: vztahy v rodině, ve třídě a ve škole; pravidla soužití a jejich vyvozování; tolerance k odlišnostem
 • Osobnostní a sociální výchova: sebepoznání a poznávání druhých, mezilidské vztahy, spolupráce a role ve skupině
@@ -3964,15 +4029,15 @@
 • Český jazyk a literatura: pravidla dialogu, střídání se v hovoru, formulace ocenění a věcného postřehu</t>
         </is>
       </c>
-      <c r="J55" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K55" s="3" t="inlineStr"/>
+      <c r="J56" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K56" s="3" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K55"/>
+  <autoFilter ref="A1:K56"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4349,17 +4414,17 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>15, 38, 48</t>
+          <t>15, 38, 48, 52</t>
         </is>
       </c>
       <c r="F10" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="11">
@@ -5213,17 +5278,17 @@
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>3, 4, 5</t>
+          <t>3, 4, 5, 52</t>
         </is>
       </c>
       <c r="F34" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H34" s="3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="35">
@@ -5424,7 +5489,7 @@
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>52</t>
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr">
@@ -5433,13 +5498,13 @@
         </is>
       </c>
       <c r="F40" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G40" s="3" t="n">
         <v>1</v>
       </c>
       <c r="H40" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="41">
@@ -7553,17 +7618,17 @@
       </c>
       <c r="E99" s="3" t="inlineStr">
         <is>
-          <t>2, 39</t>
+          <t>2, 39, 52</t>
         </is>
       </c>
       <c r="F99" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G99" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H99" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="100">
@@ -7661,17 +7726,17 @@
       </c>
       <c r="E102" s="3" t="inlineStr">
         <is>
-          <t>7, 19, 27, 29, 36</t>
+          <t>7, 19, 27, 29, 36, 52</t>
         </is>
       </c>
       <c r="F102" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G102" s="3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H102" s="3" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="103">
@@ -7769,17 +7834,17 @@
       </c>
       <c r="E105" s="3" t="inlineStr">
         <is>
-          <t>18, 46</t>
+          <t>18, 46, 52</t>
         </is>
       </c>
       <c r="F105" s="3" t="n">
         <v>2</v>
       </c>
       <c r="G105" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H105" s="3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="106">
@@ -7908,7 +7973,7 @@
       </c>
       <c r="D109" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>52</t>
         </is>
       </c>
       <c r="E109" s="3" t="inlineStr">
@@ -7917,13 +7982,13 @@
         </is>
       </c>
       <c r="F109" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G109" s="3" t="n">
         <v>2</v>
       </c>
       <c r="H109" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="110">

</xml_diff>